<commit_message>
Run analyses with round 11 included for RQ1, RQ2 and exploratory results
</commit_message>
<xml_diff>
--- a/results/cntry_desc_tbl.xlsx
+++ b/results/cntry_desc_tbl.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -433,19 +433,19 @@
         </is>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2">
-        <v>11869</v>
+        <v>14032</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -455,22 +455,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.51</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>60433</t>
+          <t>60613</t>
         </is>
       </c>
     </row>
@@ -501,14 +501,14 @@
         </is>
       </c>
       <c r="B3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3">
-        <v>15312</v>
+        <v>16681</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-0.04</t>
+          <t>-0.03</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -533,12 +533,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.87</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>0.38</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>56803</t>
+          <t>57081</t>
         </is>
       </c>
     </row>
@@ -569,14 +569,14 @@
         </is>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4">
-        <v>11429</v>
+        <v>13437</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.04</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.19</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -596,37 +596,37 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0.46</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.78</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0.72</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0.45</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>0.78</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0.72</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>23096</t>
+          <t>23553</t>
         </is>
       </c>
     </row>
@@ -637,10 +637,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>14723</v>
+        <v>15914</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -649,12 +649,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.87</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.84</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>74937</t>
+          <t>75272</t>
         </is>
       </c>
     </row>
@@ -705,10 +705,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>4116</v>
+        <v>4580</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -717,12 +717,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>-0.44</t>
+          <t>-0.46</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -732,22 +732,22 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>-0.16</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.78</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>41998</t>
+          <t>42461</t>
         </is>
       </c>
     </row>
@@ -776,11 +776,11 @@
         <v>9</v>
       </c>
       <c r="C7">
-        <v>17101</v>
+        <v>17085</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.14</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.71</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>40528</t>
+          <t>40845</t>
         </is>
       </c>
     </row>
@@ -841,14 +841,14 @@
         </is>
       </c>
       <c r="B8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8">
-        <v>23579</v>
+        <v>25753</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>-0.47</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>57203</t>
+          <t>57452</t>
         </is>
       </c>
     </row>
@@ -912,48 +912,48 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>10594</v>
+        <v>10590</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-0.14</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0.48</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>0.96</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>-0.17</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0.92</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0.31</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.94</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>0.49</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>0.96</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>0.77</t>
@@ -966,7 +966,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>62482</t>
+          <t>62890</t>
         </is>
       </c>
     </row>
@@ -977,10 +977,10 @@
         </is>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10">
-        <v>14874</v>
+        <v>15958</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -994,17 +994,17 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-0.33</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>35133</t>
+          <t>35432</t>
         </is>
       </c>
     </row>
@@ -1045,14 +1045,14 @@
         </is>
       </c>
       <c r="B11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11">
-        <v>15164</v>
+        <v>16795</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.63</t>
+          <t>-0.65</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1072,17 +1072,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>-0.27</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.97</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>43543</t>
+          <t>43715</t>
         </is>
       </c>
     </row>
@@ -1113,14 +1113,14 @@
         </is>
       </c>
       <c r="B12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12">
-        <v>16055</v>
+        <v>17394</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.56</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>54215</t>
+          <t>54307</t>
         </is>
       </c>
     </row>
@@ -1181,14 +1181,14 @@
         </is>
       </c>
       <c r="B13">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13">
-        <v>16705</v>
+        <v>18277</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1208,17 +1208,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>-0.03</t>
+          <t>-0.05</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>50086</t>
+          <t>50265</t>
         </is>
       </c>
     </row>
@@ -1249,14 +1249,14 @@
         </is>
       </c>
       <c r="B14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C14">
-        <v>19291</v>
+        <v>20697</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.14</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.38</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>48851</t>
+          <t>49017</t>
         </is>
       </c>
     </row>
@@ -1317,39 +1317,39 @@
         </is>
       </c>
       <c r="B15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15">
-        <v>11454</v>
+        <v>13982</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.09</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-0.06</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>35026</t>
+          <t>35109</t>
         </is>
       </c>
     </row>
@@ -1385,49 +1385,49 @@
         </is>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16">
-        <v>5563</v>
+        <v>6895</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.24</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>-0.42</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>1.09</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>-0.41</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>-0.02</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>0.87</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>30327</t>
+          <t>30818</t>
         </is>
       </c>
     </row>
@@ -1453,24 +1453,24 @@
         </is>
       </c>
       <c r="B17">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17">
-        <v>13942</v>
+        <v>15877</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1480,37 +1480,37 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.36</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>0.32</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>0.99</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>0.32</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>0.68</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>0.99</t>
-        </is>
-      </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>30903</t>
+          <t>31333</t>
         </is>
       </c>
     </row>
@@ -1521,19 +1521,19 @@
         </is>
       </c>
       <c r="B18">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C18">
-        <v>18573</v>
+        <v>20405</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>-0.00</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>75379</t>
+          <t>77203</t>
         </is>
       </c>
     </row>
@@ -1589,14 +1589,14 @@
         </is>
       </c>
       <c r="B19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19">
-        <v>12749</v>
+        <v>13446</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.14</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1616,37 +1616,37 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.45</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>0.29</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>0.87</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0.71</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
           <t>0.97</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>0.29</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>0.87</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>0.71</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>0.97</t>
-        </is>
-      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>39179</t>
+          <t>39558</t>
         </is>
       </c>
     </row>
@@ -1657,14 +1657,14 @@
         </is>
       </c>
       <c r="B20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C20">
-        <v>2830</v>
+        <v>3446</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>-0.34</t>
+          <t>-0.31</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1674,34 +1674,34 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>-0.58</t>
+          <t>-0.54</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.91</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>0.91</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>0.47</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>0.92</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>0.48</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>0.92</t>
-        </is>
-      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>0.86</t>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>58455</t>
+          <t>58852</t>
         </is>
       </c>
     </row>
@@ -1725,34 +1725,34 @@
         </is>
       </c>
       <c r="B21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21">
-        <v>7871</v>
+        <v>10458</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.09</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-0.06</t>
+          <t>-0.03</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>49623</t>
+          <t>49764</t>
         </is>
       </c>
     </row>
@@ -1793,44 +1793,44 @@
         </is>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C22">
-        <v>10453</v>
+        <v>11541</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0.77</t>
+          <t>0.76</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>0.45</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>32397</t>
+          <t>33023</t>
         </is>
       </c>
     </row>
@@ -1861,24 +1861,24 @@
         </is>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C23">
-        <v>2425</v>
+        <v>3458</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>-0.03</t>
+          <t>-0.05</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1888,17 +1888,17 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>0.52</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1913,12 +1913,12 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>28443</t>
+          <t>28914</t>
         </is>
       </c>
     </row>
@@ -1929,44 +1929,44 @@
         </is>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24">
-        <v>2063</v>
+        <v>3422</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.54</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.37</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>20093</t>
+          <t>20409</t>
         </is>
       </c>
     </row>
@@ -1997,19 +1997,19 @@
         </is>
       </c>
       <c r="B25">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C25">
-        <v>16032</v>
+        <v>17478</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>0.22</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2019,22 +2019,22 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>0.87</t>
+          <t>0.86</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>62746</t>
+          <t>63106</t>
         </is>
       </c>
     </row>
@@ -2065,14 +2065,14 @@
         </is>
       </c>
       <c r="B26">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C26">
-        <v>13214</v>
+        <v>14317</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2082,17 +2082,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.14</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>85116</t>
+          <t>85342</t>
         </is>
       </c>
     </row>
@@ -2133,14 +2133,14 @@
         </is>
       </c>
       <c r="B27">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C27">
-        <v>13526</v>
+        <v>14740</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>-0.21</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>29545</t>
+          <t>30188</t>
         </is>
       </c>
     </row>
@@ -2201,102 +2201,102 @@
         </is>
       </c>
       <c r="B28">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C28">
-        <v>15713</v>
+        <v>16831</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>-0.09</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
           <t>0.98</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>-0.10</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>0.22</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>0.89</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
         <is>
           <t>0.99</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>0.20</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>0.94</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>0.30</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>0.88</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>0.73</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>0.99</t>
-        </is>
-      </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>36804</t>
+          <t>37021</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B29">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C29">
-        <v>11101</v>
+        <v>3096</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.32</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>-0.55</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2306,367 +2306,435 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.84</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0.70</t>
+          <t>0.74</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>33173</t>
+          <t>18507</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="B30">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C30">
-        <v>13036</v>
+        <v>11105</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>-0.21</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.96</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0.29</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>0.96</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>0.70</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>56811</t>
+          <t>33478</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B31">
         <v>10</v>
       </c>
       <c r="C31">
-        <v>11237</v>
+        <v>14058</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0.87</t>
+          <t>0.96</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.96</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>0.41</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>0.96</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>39154</t>
+          <t>57085</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="B32">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C32">
-        <v>9655</v>
+        <v>12254</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>0.87</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>-0.05</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>0.86</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.37</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>0.45</t>
+          <t>0.42</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.91</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0.69</t>
+          <t>0.74</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>30472</t>
+          <t>39550</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B33">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C33">
-        <v>3701</v>
+        <v>10905</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>0.29</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>0.52</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>0.69</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>22856</t>
+          <t>30882</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34">
+        <v>3704</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0.41</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>0.29</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>0.53</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>0.63</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0.61</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>0.90</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>23375</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Ukraine</t>
         </is>
       </c>
-      <c r="B34">
-        <v>5</v>
-      </c>
-      <c r="C34">
-        <v>8420</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>0.22</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>1.21</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>0.40</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>0.32</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
+      <c r="B35">
+        <v>6</v>
+      </c>
+      <c r="C35">
+        <v>10778</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>1.22</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>0.39</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>0.37</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t>NaN</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>0.70</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>16407</t>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>16385</t>
         </is>
       </c>
     </row>

</xml_diff>